<commit_message>
all runs and statistics
</commit_message>
<xml_diff>
--- a/results/03_crf_transitions_mined.xlsx
+++ b/results/03_crf_transitions_mined.xlsx
@@ -557,67 +557,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>43.13</v>
+        <v>45.1</v>
       </c>
       <c r="C4" t="n">
-        <v>51.17</v>
+        <v>48.46</v>
       </c>
       <c r="D4" t="n">
-        <v>39.79</v>
+        <v>43.97</v>
       </c>
       <c r="E4" t="n">
-        <v>95.14</v>
+        <v>95.29000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>95.02</v>
+        <v>95.18000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>95.39</v>
+        <v>95.5</v>
       </c>
       <c r="H4" t="n">
-        <v>95.39</v>
+        <v>95.5</v>
       </c>
       <c r="I4" t="n">
-        <v>35.91</v>
+        <v>45.61</v>
       </c>
       <c r="J4" t="n">
-        <v>42.31</v>
+        <v>49.84</v>
       </c>
       <c r="K4" t="n">
-        <v>33.76</v>
+        <v>48.97</v>
       </c>
       <c r="L4" t="n">
-        <v>95.75</v>
+        <v>95.84</v>
       </c>
       <c r="M4" t="n">
-        <v>95.81999999999999</v>
+        <v>95.92</v>
       </c>
       <c r="N4" t="n">
-        <v>95.91</v>
+        <v>95.95999999999999</v>
       </c>
       <c r="O4" t="n">
-        <v>95.91</v>
+        <v>95.95999999999999</v>
       </c>
       <c r="P4" t="n">
-        <v>50.34</v>
+        <v>50.85</v>
       </c>
       <c r="Q4" t="n">
-        <v>56.64</v>
+        <v>53.26</v>
       </c>
       <c r="R4" t="n">
-        <v>49.98</v>
+        <v>50.86</v>
       </c>
       <c r="S4" t="n">
-        <v>96.90000000000001</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="T4" t="n">
-        <v>96.98</v>
+        <v>97.20999999999999</v>
       </c>
       <c r="U4" t="n">
-        <v>96.95999999999999</v>
+        <v>97.25</v>
       </c>
       <c r="V4" t="n">
-        <v>96.95999999999999</v>
+        <v>97.25</v>
       </c>
     </row>
   </sheetData>
@@ -744,13 +744,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.22</v>
+        <v>31.67</v>
       </c>
       <c r="D4" t="n">
-        <v>39.53</v>
+        <v>42.68</v>
       </c>
       <c r="E4" t="n">
-        <v>24.46</v>
+        <v>25.18</v>
       </c>
       <c r="F4" t="n">
         <v>139</v>
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>40</v>
+        <v>45.36</v>
       </c>
       <c r="D5" t="n">
-        <v>44.9</v>
+        <v>61.11</v>
       </c>
       <c r="E5" t="n">
         <v>36.07</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>23.53</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>21.05</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>26.67</v>
       </c>
       <c r="F6" t="n">
         <v>15</v>
@@ -876,34 +876,34 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>52.28</v>
+        <v>53.99</v>
       </c>
       <c r="D8" t="n">
-        <v>65.48999999999999</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>43.51</v>
+        <v>46.26</v>
       </c>
       <c r="F8" t="n">
         <v>1749</v>
       </c>
       <c r="G8" t="n">
-        <v>68.53</v>
+        <v>68.91</v>
       </c>
       <c r="H8" t="n">
-        <v>87.76000000000001</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>56.22</v>
+        <v>58.11</v>
       </c>
       <c r="J8" t="n">
         <v>370</v>
       </c>
       <c r="K8" t="n">
-        <v>51.43</v>
+        <v>56.25</v>
       </c>
       <c r="L8" t="n">
-        <v>52.94</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="M8" t="n">
         <v>50</v>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25.81</v>
+        <v>24.62</v>
       </c>
       <c r="D9" t="n">
-        <v>36.36</v>
+        <v>32</v>
       </c>
       <c r="E9" t="n">
         <v>20</v>
@@ -931,13 +931,13 @@
         <v>40</v>
       </c>
       <c r="G9" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
       <c r="H9" t="n">
-        <v>33.33</v>
+        <v>66.67</v>
       </c>
       <c r="I9" t="n">
-        <v>9.09</v>
+        <v>18.18</v>
       </c>
       <c r="J9" t="n">
         <v>11</v>
@@ -1024,34 +1024,34 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>55.52</v>
+        <v>57.62</v>
       </c>
       <c r="D12" t="n">
-        <v>66.67</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>47.57</v>
+        <v>50.49</v>
       </c>
       <c r="F12" t="n">
         <v>206</v>
       </c>
       <c r="G12" t="n">
-        <v>46.91</v>
+        <v>50.63</v>
       </c>
       <c r="H12" t="n">
-        <v>76</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>33.93</v>
+        <v>35.71</v>
       </c>
       <c r="J12" t="n">
         <v>56</v>
       </c>
       <c r="K12" t="n">
-        <v>40</v>
+        <v>33.33</v>
       </c>
       <c r="L12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M12" t="n">
         <v>25</v>
@@ -1067,25 +1067,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>59.7</v>
+        <v>47.06</v>
       </c>
       <c r="D13" t="n">
-        <v>57.14</v>
+        <v>44.44</v>
       </c>
       <c r="E13" t="n">
-        <v>62.5</v>
+        <v>50</v>
       </c>
       <c r="F13" t="n">
         <v>32</v>
       </c>
       <c r="G13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H13" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I13" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="J13" t="n">
         <v>4</v>
@@ -1110,34 +1110,34 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>49.69</v>
+        <v>51.13</v>
       </c>
       <c r="D14" t="n">
-        <v>57.97</v>
+        <v>57.24</v>
       </c>
       <c r="E14" t="n">
-        <v>43.48</v>
+        <v>46.2</v>
       </c>
       <c r="F14" t="n">
         <v>368</v>
       </c>
       <c r="G14" t="n">
-        <v>61.25</v>
+        <v>59.17</v>
       </c>
       <c r="H14" t="n">
-        <v>58.33</v>
+        <v>53.76</v>
       </c>
       <c r="I14" t="n">
-        <v>64.47</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>76</v>
       </c>
       <c r="K14" t="n">
-        <v>28.57</v>
+        <v>33.33</v>
       </c>
       <c r="L14" t="n">
-        <v>18.18</v>
+        <v>22.22</v>
       </c>
       <c r="M14" t="n">
         <v>66.67</v>
@@ -1156,22 +1156,22 @@
         <v>33.33</v>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>28.57</v>
       </c>
       <c r="E15" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F15" t="n">
         <v>10</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>28.57</v>
       </c>
       <c r="J15" t="n">
         <v>7</v>
@@ -1188,37 +1188,37 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>90.51000000000001</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>89.37</v>
+        <v>89.81</v>
       </c>
       <c r="E16" t="n">
-        <v>91.68000000000001</v>
+        <v>92.2</v>
       </c>
       <c r="F16" t="n">
         <v>12166</v>
       </c>
       <c r="G16" t="n">
-        <v>90.81</v>
+        <v>91.33</v>
       </c>
       <c r="H16" t="n">
-        <v>91.17</v>
+        <v>91.59</v>
       </c>
       <c r="I16" t="n">
-        <v>90.44</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="J16" t="n">
         <v>1758</v>
       </c>
       <c r="K16" t="n">
-        <v>90.42</v>
+        <v>91.3</v>
       </c>
       <c r="L16" t="n">
-        <v>88.73999999999999</v>
+        <v>89.94</v>
       </c>
       <c r="M16" t="n">
-        <v>92.16</v>
+        <v>92.72</v>
       </c>
       <c r="N16" t="n">
         <v>906</v>
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22.78</v>
+        <v>30.23</v>
       </c>
       <c r="D17" t="n">
-        <v>52.94</v>
+        <v>54.17</v>
       </c>
       <c r="E17" t="n">
-        <v>14.52</v>
+        <v>20.97</v>
       </c>
       <c r="F17" t="n">
         <v>62</v>
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>70.36</v>
+        <v>71.53</v>
       </c>
       <c r="D18" t="n">
-        <v>76.06</v>
+        <v>77.01000000000001</v>
       </c>
       <c r="E18" t="n">
-        <v>65.45</v>
+        <v>66.78</v>
       </c>
       <c r="F18" t="n">
         <v>301</v>
@@ -1290,10 +1290,10 @@
         <v>8</v>
       </c>
       <c r="K18" t="n">
-        <v>66.67</v>
+        <v>50</v>
       </c>
       <c r="L18" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M18" t="n">
         <v>50</v>
@@ -1309,37 +1309,37 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>52.23</v>
+        <v>52.3</v>
       </c>
       <c r="D19" t="n">
-        <v>61.03</v>
+        <v>62.79</v>
       </c>
       <c r="E19" t="n">
-        <v>45.64</v>
+        <v>44.81</v>
       </c>
       <c r="F19" t="n">
         <v>1194</v>
       </c>
       <c r="G19" t="n">
-        <v>71.29000000000001</v>
+        <v>70.93000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>71.52</v>
+        <v>72.08</v>
       </c>
       <c r="I19" t="n">
-        <v>71.06999999999999</v>
+        <v>69.81</v>
       </c>
       <c r="J19" t="n">
         <v>159</v>
       </c>
       <c r="K19" t="n">
-        <v>56.41</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>80.48999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="M19" t="n">
-        <v>43.42</v>
+        <v>52.63</v>
       </c>
       <c r="N19" t="n">
         <v>76</v>
@@ -1352,25 +1352,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>13.33</v>
+        <v>17.02</v>
       </c>
       <c r="D20" t="n">
-        <v>40</v>
+        <v>18.18</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F20" t="n">
         <v>25</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>36.36</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>28.57</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J20" t="n">
         <v>4</v>
@@ -1395,37 +1395,37 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>93.28</v>
+        <v>93.41</v>
       </c>
       <c r="D21" t="n">
-        <v>91.40000000000001</v>
+        <v>91.95</v>
       </c>
       <c r="E21" t="n">
-        <v>95.23999999999999</v>
+        <v>94.91</v>
       </c>
       <c r="F21" t="n">
         <v>7668</v>
       </c>
       <c r="G21" t="n">
-        <v>95.34</v>
+        <v>95.09</v>
       </c>
       <c r="H21" t="n">
-        <v>93.98999999999999</v>
+        <v>94.29000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>96.72</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="J21" t="n">
         <v>1342</v>
       </c>
       <c r="K21" t="n">
-        <v>97.39</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>96.98</v>
+        <v>96.84</v>
       </c>
       <c r="M21" t="n">
-        <v>97.8</v>
+        <v>98.31</v>
       </c>
       <c r="N21" t="n">
         <v>592</v>
@@ -1438,13 +1438,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49.54</v>
+        <v>53.16</v>
       </c>
       <c r="D22" t="n">
-        <v>60.67</v>
+        <v>58.33</v>
       </c>
       <c r="E22" t="n">
-        <v>41.86</v>
+        <v>48.84</v>
       </c>
       <c r="F22" t="n">
         <v>129</v>
@@ -1473,13 +1473,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.64</v>
+        <v>72.42</v>
       </c>
       <c r="D23" t="n">
-        <v>77.45</v>
+        <v>78.06</v>
       </c>
       <c r="E23" t="n">
-        <v>70.19</v>
+        <v>67.55</v>
       </c>
       <c r="F23" t="n">
         <v>416</v>
@@ -1500,37 +1500,37 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>52.46</v>
+        <v>52.77</v>
       </c>
       <c r="D24" t="n">
-        <v>55.18</v>
+        <v>55.11</v>
       </c>
       <c r="E24" t="n">
-        <v>50</v>
+        <v>50.61</v>
       </c>
       <c r="F24" t="n">
         <v>490</v>
       </c>
       <c r="G24" t="n">
-        <v>36.59</v>
+        <v>35.9</v>
       </c>
       <c r="H24" t="n">
-        <v>34.88</v>
+        <v>35.9</v>
       </c>
       <c r="I24" t="n">
-        <v>38.46</v>
+        <v>35.9</v>
       </c>
       <c r="J24" t="n">
         <v>39</v>
       </c>
       <c r="K24" t="n">
-        <v>52.17</v>
+        <v>61.9</v>
       </c>
       <c r="L24" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="M24" t="n">
-        <v>54.55</v>
+        <v>59.09</v>
       </c>
       <c r="N24" t="n">
         <v>22</v>
@@ -1543,25 +1543,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>57.36</v>
+        <v>62.9</v>
       </c>
       <c r="D25" t="n">
-        <v>54.81</v>
+        <v>55.62</v>
       </c>
       <c r="E25" t="n">
-        <v>60.16</v>
+        <v>72.36</v>
       </c>
       <c r="F25" t="n">
         <v>123</v>
       </c>
       <c r="G25" t="n">
-        <v>47.37</v>
+        <v>61.54</v>
       </c>
       <c r="H25" t="n">
-        <v>50</v>
+        <v>63.16</v>
       </c>
       <c r="I25" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J25" t="n">
         <v>20</v>
@@ -1578,25 +1578,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18.75</v>
+        <v>16.9</v>
       </c>
       <c r="D26" t="n">
-        <v>23.08</v>
+        <v>25.53</v>
       </c>
       <c r="E26" t="n">
-        <v>15.79</v>
+        <v>12.63</v>
       </c>
       <c r="F26" t="n">
         <v>95</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>9.09</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>33.33</v>
       </c>
       <c r="J26" t="n">
         <v>3</v>
@@ -1621,34 +1621,34 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>64.44</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D27" t="n">
-        <v>62.46</v>
+        <v>66.56</v>
       </c>
       <c r="E27" t="n">
-        <v>66.56</v>
+        <v>69.18000000000001</v>
       </c>
       <c r="F27" t="n">
         <v>305</v>
       </c>
       <c r="G27" t="n">
-        <v>76.70999999999999</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>70</v>
+        <v>66.67</v>
       </c>
       <c r="I27" t="n">
-        <v>84.84999999999999</v>
+        <v>72.73</v>
       </c>
       <c r="J27" t="n">
         <v>33</v>
       </c>
       <c r="K27" t="n">
-        <v>74.06999999999999</v>
+        <v>76.92</v>
       </c>
       <c r="L27" t="n">
-        <v>76.92</v>
+        <v>83.33</v>
       </c>
       <c r="M27" t="n">
         <v>71.43000000000001</v>
@@ -1664,13 +1664,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>55.91</v>
+        <v>61.94</v>
       </c>
       <c r="D28" t="n">
-        <v>57.35</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E28" t="n">
-        <v>54.55</v>
+        <v>58.04</v>
       </c>
       <c r="F28" t="n">
         <v>143</v>
@@ -1707,25 +1707,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>17.39</v>
+        <v>19.51</v>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>15.38</v>
       </c>
       <c r="E29" t="n">
-        <v>13.33</v>
+        <v>26.67</v>
       </c>
       <c r="F29" t="n">
         <v>15</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>33.33</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -1742,25 +1742,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30.77</v>
+        <v>33.33</v>
       </c>
       <c r="D30" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E30" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F30" t="n">
         <v>8</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>66.67</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J30" t="n">
         <v>1</v>
@@ -1777,13 +1777,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>98.27</v>
+        <v>98.31</v>
       </c>
       <c r="D31" t="n">
-        <v>97.91</v>
+        <v>97.98999999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>98.63</v>
+        <v>98.64</v>
       </c>
       <c r="F31" t="n">
         <v>101885</v>
@@ -1792,22 +1792,22 @@
         <v>98.29000000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>97.83</v>
+        <v>97.87</v>
       </c>
       <c r="I31" t="n">
-        <v>98.75</v>
+        <v>98.72</v>
       </c>
       <c r="J31" t="n">
         <v>14471</v>
       </c>
       <c r="K31" t="n">
-        <v>98.66</v>
+        <v>98.75</v>
       </c>
       <c r="L31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.75</v>
       </c>
       <c r="M31" t="n">
-        <v>98.62</v>
+        <v>98.73999999999999</v>
       </c>
       <c r="N31" t="n">
         <v>6815</v>

</xml_diff>